<commit_message>
seo: fix titles, descriptions und schema auf allen Seiten
- Titel-Suffix von '– Daniel Eck – Versicherungsmakler' auf '| Eck Versicherung' geändert (116 Dateien)
- 25 verbleibende zu lange Blog-Titel auf ≤60 Zeichen gekürzt
- 67 Meta-Descriptions von >160 auf ≤156 Zeichen gekürzt
- InsuranceAgency JSON-LD Schema auf 118 Hauptseiten hinzugefügt (war nur auf start.html)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bkv-kampagne/kontakte_neu.xlsx
+++ b/bkv-kampagne/kontakte_neu.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x15 xr xr6 xr10">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\danie\Webseite_Eckversicherung\bkv-kampagne\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C9532C57-5CDA-4D14-A55B-7D2B33AF0D7E}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26720909-033D-42A8-98F0-A22DD8D4E30C}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="10800"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="10284" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="kontakte" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="292" uniqueCount="193">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="326" uniqueCount="193">
   <si>
     <t>Anrede</t>
   </si>
@@ -136,9 +136,6 @@
     <t>Untermaßfeld</t>
   </si>
   <si>
-    <t>Personalabteilung</t>
-  </si>
-  <si>
     <t>Werra Papier Wernshausen GmbH</t>
   </si>
   <si>
@@ -250,7 +247,7 @@
     <t>Julia</t>
   </si>
   <si>
-    <t>NillerPersonal</t>
+    <t>Niller</t>
   </si>
   <si>
     <t>Ehrhardt AG</t>
@@ -289,18 +286,9 @@
     <t>info@qsil.de</t>
   </si>
   <si>
-    <t>Josse</t>
-  </si>
-  <si>
-    <t>Coudré</t>
-  </si>
-  <si>
     <t>Sandvik Tooling Supply Germany</t>
   </si>
   <si>
-    <t>support.coromant@sandvik.com</t>
-  </si>
-  <si>
     <t>Paragon Electronic GmbH</t>
   </si>
   <si>
@@ -529,10 +517,10 @@
     <t>info@analytics-thueringen.de</t>
   </si>
   <si>
-    <t>Uwe</t>
-  </si>
-  <si>
-    <t>Kleemann</t>
+    <t>Denise</t>
+  </si>
+  <si>
+    <t>Reese</t>
   </si>
   <si>
     <t>alupress GmbH</t>
@@ -598,14 +586,26 @@
     <t>info@dytb-thueringen.de</t>
   </si>
   <si>
-    <t>SWZ Zella-Mehlis (Rennsteig-Gruppe)</t>
+    <t>Franziska</t>
+  </si>
+  <si>
+    <t>Huhn</t>
+  </si>
+  <si>
+    <t>franziska.huhn@sandvik.com</t>
+  </si>
+  <si>
+    <t>falsches Konto</t>
+  </si>
+  <si>
+    <t>richtiges Konto</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="18" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -740,8 +740,16 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="33">
+  <fills count="35">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -919,6 +927,18 @@
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.39997558519241921"/>
         <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -1038,7 +1058,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="42">
+  <cellStyleXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
@@ -1081,11 +1101,23 @@
     <xf numFmtId="0" fontId="1" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="42"/>
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="42">
+  <cellStyles count="43">
     <cellStyle name="20 % - Akzent1" xfId="19" builtinId="30" customBuiltin="1"/>
     <cellStyle name="20 % - Akzent2" xfId="23" builtinId="34" customBuiltin="1"/>
     <cellStyle name="20 % - Akzent3" xfId="27" builtinId="38" customBuiltin="1"/>
@@ -1116,6 +1148,7 @@
     <cellStyle name="Ergebnis" xfId="17" builtinId="25" customBuiltin="1"/>
     <cellStyle name="Erklärender Text" xfId="16" builtinId="53" customBuiltin="1"/>
     <cellStyle name="Gut" xfId="6" builtinId="26" customBuiltin="1"/>
+    <cellStyle name="Link" xfId="42" builtinId="8"/>
     <cellStyle name="Neutral" xfId="8" builtinId="28" customBuiltin="1"/>
     <cellStyle name="Notiz" xfId="15" builtinId="10" customBuiltin="1"/>
     <cellStyle name="Schlecht" xfId="7" builtinId="27" customBuiltin="1"/>
@@ -1438,15 +1471,16 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H44"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:K44"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="44.88671875" customWidth="1"/>
-    <col min="3" max="3" width="33.77734375" customWidth="1"/>
+    <col min="1" max="1" width="38.5546875" customWidth="1"/>
+    <col min="4" max="4" width="34.44140625" customWidth="1"/>
+    <col min="6" max="6" width="31.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1472,7 +1506,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -1491,8 +1525,12 @@
       <c r="H2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="J2" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="K2" s="3"/>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>13</v>
       </c>
@@ -1517,8 +1555,12 @@
       <c r="H3" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="J3" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="K3" s="3"/>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>20</v>
       </c>
@@ -1543,10 +1585,14 @@
       <c r="H4" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="J4" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="K4" s="3"/>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="B5" t="s">
         <v>27</v>
@@ -1569,8 +1615,12 @@
       <c r="H5" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="J5" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="K5" s="3"/>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>13</v>
       </c>
@@ -1595,94 +1645,107 @@
       <c r="H6" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="J6" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="K6" s="3"/>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>13</v>
       </c>
-      <c r="B7" t="s">
+      <c r="D7" t="s">
         <v>38</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7" t="s">
         <v>39</v>
       </c>
-      <c r="E7" t="s">
+      <c r="F7" t="s">
         <v>40</v>
-      </c>
-      <c r="F7" t="s">
-        <v>41</v>
       </c>
       <c r="G7">
         <v>800</v>
       </c>
       <c r="H7" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+        <v>41</v>
+      </c>
+      <c r="J7" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="K7" s="3"/>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>13</v>
       </c>
       <c r="B8" t="s">
+        <v>42</v>
+      </c>
+      <c r="C8" t="s">
         <v>43</v>
       </c>
-      <c r="C8" t="s">
+      <c r="D8" t="s">
         <v>44</v>
-      </c>
-      <c r="D8" t="s">
-        <v>45</v>
       </c>
       <c r="E8" t="s">
         <v>35</v>
       </c>
       <c r="F8" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="G8">
         <v>690</v>
       </c>
       <c r="H8" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+        <v>46</v>
+      </c>
+      <c r="J8" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="K8" s="3"/>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>8</v>
       </c>
       <c r="D9" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E9" t="s">
         <v>35</v>
       </c>
       <c r="F9" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G9">
         <v>680</v>
       </c>
       <c r="H9" t="s">
+        <v>49</v>
+      </c>
+      <c r="J9" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="K9" s="3"/>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>20</v>
+      </c>
+      <c r="B10" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>13</v>
-      </c>
-      <c r="B10" t="s">
+      <c r="C10" t="s">
         <v>51</v>
       </c>
-      <c r="C10" t="s">
+      <c r="D10" t="s">
         <v>52</v>
       </c>
-      <c r="D10" t="s">
+      <c r="E10" t="s">
         <v>53</v>
       </c>
-      <c r="E10" t="s">
+      <c r="F10" t="s">
         <v>54</v>
-      </c>
-      <c r="F10" t="s">
-        <v>55</v>
       </c>
       <c r="G10">
         <v>650</v>
@@ -1690,25 +1753,29 @@
       <c r="H10" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="J10" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="K10" s="3"/>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="B11" t="s">
+        <v>55</v>
+      </c>
+      <c r="C11" t="s">
         <v>56</v>
       </c>
-      <c r="C11" t="s">
+      <c r="D11" t="s">
         <v>57</v>
       </c>
-      <c r="D11" t="s">
+      <c r="E11" t="s">
         <v>58</v>
       </c>
-      <c r="E11" t="s">
+      <c r="F11" t="s">
         <v>59</v>
-      </c>
-      <c r="F11" t="s">
-        <v>60</v>
       </c>
       <c r="G11">
         <v>575</v>
@@ -1716,25 +1783,29 @@
       <c r="H11" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="J11" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="K11" s="3"/>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>13</v>
       </c>
       <c r="B12" t="s">
+        <v>60</v>
+      </c>
+      <c r="C12" t="s">
         <v>61</v>
       </c>
-      <c r="C12" t="s">
+      <c r="D12" t="s">
         <v>62</v>
-      </c>
-      <c r="D12" t="s">
-        <v>63</v>
       </c>
       <c r="E12" t="s">
         <v>35</v>
       </c>
       <c r="F12" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="G12">
         <v>400</v>
@@ -1742,25 +1813,29 @@
       <c r="H12" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="J12" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="K12" s="3"/>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>20</v>
       </c>
       <c r="B13" t="s">
+        <v>64</v>
+      </c>
+      <c r="C13" t="s">
         <v>65</v>
       </c>
-      <c r="C13" t="s">
+      <c r="D13" t="s">
         <v>66</v>
       </c>
-      <c r="D13" t="s">
+      <c r="E13" t="s">
         <v>67</v>
       </c>
-      <c r="E13" t="s">
+      <c r="F13" t="s">
         <v>68</v>
-      </c>
-      <c r="F13" t="s">
-        <v>69</v>
       </c>
       <c r="G13">
         <v>370</v>
@@ -1768,103 +1843,119 @@
       <c r="H13" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="J13" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="K13" s="3"/>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>13</v>
       </c>
       <c r="B14" t="s">
+        <v>69</v>
+      </c>
+      <c r="C14" t="s">
         <v>70</v>
       </c>
-      <c r="C14" t="s">
+      <c r="D14" t="s">
         <v>71</v>
-      </c>
-      <c r="D14" t="s">
-        <v>72</v>
       </c>
       <c r="E14" t="s">
         <v>35</v>
       </c>
       <c r="F14" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G14">
         <v>350</v>
       </c>
       <c r="H14" t="s">
+        <v>73</v>
+      </c>
+      <c r="J14" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="K14" s="3"/>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>20</v>
+      </c>
+      <c r="B15" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
-        <v>13</v>
-      </c>
-      <c r="B15" t="s">
+      <c r="C15" t="s">
         <v>75</v>
       </c>
-      <c r="C15" t="s">
+      <c r="D15" t="s">
         <v>76</v>
       </c>
-      <c r="D15" t="s">
+      <c r="E15" t="s">
         <v>77</v>
       </c>
-      <c r="E15" t="s">
+      <c r="F15" t="s">
         <v>78</v>
-      </c>
-      <c r="F15" t="s">
-        <v>79</v>
       </c>
       <c r="G15">
         <v>330</v>
       </c>
       <c r="H15" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+        <v>73</v>
+      </c>
+      <c r="J15" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="K15" s="3"/>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="B16" t="s">
+        <v>79</v>
+      </c>
+      <c r="C16" t="s">
         <v>80</v>
       </c>
-      <c r="C16" t="s">
+      <c r="D16" t="s">
         <v>81</v>
-      </c>
-      <c r="D16" t="s">
-        <v>82</v>
       </c>
       <c r="E16" t="s">
         <v>10</v>
       </c>
       <c r="F16" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="G16">
         <v>300</v>
       </c>
       <c r="H16" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+        <v>83</v>
+      </c>
+      <c r="J16" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="K16" s="3"/>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>13</v>
       </c>
       <c r="B17" t="s">
+        <v>84</v>
+      </c>
+      <c r="C17" t="s">
         <v>85</v>
       </c>
-      <c r="C17" t="s">
+      <c r="D17" t="s">
         <v>86</v>
-      </c>
-      <c r="D17" t="s">
-        <v>87</v>
       </c>
       <c r="E17" t="s">
         <v>35</v>
       </c>
       <c r="F17" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G17">
         <v>270</v>
@@ -1872,215 +1963,251 @@
       <c r="H17" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="J17" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="K17" s="3"/>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="B18" t="s">
-        <v>89</v>
+        <v>188</v>
       </c>
       <c r="C18" t="s">
-        <v>90</v>
+        <v>189</v>
       </c>
       <c r="D18" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="E18" t="s">
         <v>35</v>
       </c>
-      <c r="F18" t="s">
-        <v>92</v>
+      <c r="F18" s="1" t="s">
+        <v>190</v>
       </c>
       <c r="G18">
         <v>260</v>
       </c>
       <c r="H18" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+        <v>41</v>
+      </c>
+      <c r="J18" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="K18" s="3"/>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>8</v>
       </c>
       <c r="D19" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="E19" t="s">
         <v>35</v>
       </c>
       <c r="F19" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="G19">
         <v>250</v>
       </c>
       <c r="H19" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
+        <v>91</v>
+      </c>
+      <c r="J19" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="K19" s="3"/>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>13</v>
       </c>
       <c r="B20" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="C20" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="D20" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="E20" t="s">
         <v>35</v>
       </c>
       <c r="F20" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="G20">
         <v>250</v>
       </c>
       <c r="H20" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
+        <v>96</v>
+      </c>
+      <c r="J20" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="K20" s="3"/>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>8</v>
       </c>
       <c r="D21" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="E21" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="F21" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="G21">
         <v>240</v>
       </c>
       <c r="H21" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
+        <v>100</v>
+      </c>
+      <c r="J21" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="K21" s="3"/>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>8</v>
       </c>
       <c r="D22" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="E22" t="s">
         <v>35</v>
       </c>
       <c r="F22" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="G22">
         <v>220</v>
       </c>
       <c r="H22" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
+        <v>100</v>
+      </c>
+      <c r="J22" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="K22" s="3"/>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>13</v>
       </c>
       <c r="B23" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="C23" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="D23" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="E23" t="s">
         <v>35</v>
       </c>
       <c r="F23" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="G23">
         <v>200</v>
       </c>
       <c r="H23" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
+        <v>107</v>
+      </c>
+      <c r="J23" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="K23" s="3"/>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>13</v>
       </c>
       <c r="B24" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="C24" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="D24" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="E24" t="s">
         <v>35</v>
       </c>
       <c r="F24" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="G24">
         <v>200</v>
       </c>
       <c r="H24" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
+        <v>100</v>
+      </c>
+      <c r="J24" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="K24" s="3"/>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>13</v>
       </c>
       <c r="B25" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="C25" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="D25" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="E25" t="s">
         <v>35</v>
       </c>
       <c r="F25" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="G25">
         <v>200</v>
       </c>
       <c r="H25" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
+        <v>91</v>
+      </c>
+      <c r="J25" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="K25" s="3"/>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>20</v>
       </c>
       <c r="B26" t="s">
+        <v>116</v>
+      </c>
+      <c r="C26" t="s">
+        <v>117</v>
+      </c>
+      <c r="D26" t="s">
+        <v>118</v>
+      </c>
+      <c r="E26" t="s">
+        <v>119</v>
+      </c>
+      <c r="F26" t="s">
         <v>120</v>
-      </c>
-      <c r="C26" t="s">
-        <v>121</v>
-      </c>
-      <c r="D26" t="s">
-        <v>122</v>
-      </c>
-      <c r="E26" t="s">
-        <v>123</v>
-      </c>
-      <c r="F26" t="s">
-        <v>124</v>
       </c>
       <c r="G26">
         <v>160</v>
@@ -2088,25 +2215,29 @@
       <c r="H26" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="J26" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="K26" s="3"/>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>20</v>
       </c>
       <c r="B27" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="C27" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="D27" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="E27" t="s">
         <v>24</v>
       </c>
       <c r="F27" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="G27">
         <v>150</v>
@@ -2114,123 +2245,143 @@
       <c r="H27" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="J27" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="K27" s="3"/>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>13</v>
       </c>
       <c r="B28" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="C28" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="D28" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="E28" t="s">
         <v>35</v>
       </c>
       <c r="F28" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="G28">
         <v>150</v>
       </c>
       <c r="H28" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
+        <v>129</v>
+      </c>
+      <c r="J28" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="K28" s="3"/>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>13</v>
       </c>
       <c r="B29" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="C29" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="D29" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="E29" t="s">
         <v>35</v>
       </c>
-      <c r="F29" t="s">
-        <v>137</v>
+      <c r="F29" s="4" t="s">
+        <v>133</v>
       </c>
       <c r="G29">
         <v>130</v>
       </c>
       <c r="H29" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
+        <v>129</v>
+      </c>
+      <c r="J29" s="5" t="s">
+        <v>192</v>
+      </c>
+      <c r="K29" s="5"/>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>8</v>
       </c>
       <c r="D30" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="E30" t="s">
         <v>35</v>
       </c>
       <c r="F30" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="G30">
         <v>120</v>
       </c>
       <c r="H30" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
+        <v>91</v>
+      </c>
+      <c r="J30" s="5" t="s">
+        <v>192</v>
+      </c>
+      <c r="K30" s="5"/>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>20</v>
       </c>
       <c r="B31" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="C31" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="D31" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="E31" t="s">
         <v>24</v>
       </c>
-      <c r="F31" t="s">
-        <v>143</v>
+      <c r="F31" s="4" t="s">
+        <v>139</v>
       </c>
       <c r="G31">
         <v>120</v>
       </c>
       <c r="H31" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
+        <v>140</v>
+      </c>
+      <c r="J31" s="5" t="s">
+        <v>192</v>
+      </c>
+      <c r="K31" s="5"/>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>13</v>
       </c>
       <c r="B32" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="C32" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="D32" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="E32" t="s">
         <v>35</v>
       </c>
-      <c r="F32" t="s">
-        <v>148</v>
+      <c r="F32" s="4" t="s">
+        <v>144</v>
       </c>
       <c r="G32">
         <v>110</v>
@@ -2238,25 +2389,29 @@
       <c r="H32" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="J32" s="5" t="s">
+        <v>192</v>
+      </c>
+      <c r="K32" s="5"/>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>13</v>
       </c>
       <c r="B33" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="C33" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="D33" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="E33" t="s">
         <v>35</v>
       </c>
-      <c r="F33" t="s">
-        <v>151</v>
+      <c r="F33" s="4" t="s">
+        <v>147</v>
       </c>
       <c r="G33">
         <v>110</v>
@@ -2264,51 +2419,59 @@
       <c r="H33" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="J33" s="5" t="s">
+        <v>192</v>
+      </c>
+      <c r="K33" s="5"/>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>13</v>
       </c>
       <c r="B34" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="C34" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="D34" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="E34" t="s">
         <v>35</v>
       </c>
-      <c r="F34" t="s">
-        <v>155</v>
+      <c r="F34" s="4" t="s">
+        <v>151</v>
       </c>
       <c r="G34">
         <v>100</v>
       </c>
       <c r="H34" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.3">
+        <v>129</v>
+      </c>
+      <c r="J34" s="5" t="s">
+        <v>192</v>
+      </c>
+      <c r="K34" s="5"/>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>13</v>
       </c>
       <c r="B35" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="C35" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="D35" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="E35" t="s">
         <v>35</v>
       </c>
-      <c r="F35" t="s">
-        <v>159</v>
+      <c r="F35" s="4" t="s">
+        <v>155</v>
       </c>
       <c r="G35">
         <v>100</v>
@@ -2316,123 +2479,143 @@
       <c r="H35" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="J35" s="5" t="s">
+        <v>192</v>
+      </c>
+      <c r="K35" s="5"/>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>13</v>
       </c>
       <c r="B36" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="C36" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="D36" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="E36" t="s">
         <v>35</v>
       </c>
-      <c r="F36" t="s">
-        <v>163</v>
+      <c r="F36" s="4" t="s">
+        <v>159</v>
       </c>
       <c r="G36">
         <v>95</v>
       </c>
       <c r="H36" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.3">
+        <v>160</v>
+      </c>
+      <c r="J36" s="5" t="s">
+        <v>192</v>
+      </c>
+      <c r="K36" s="5"/>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>13</v>
       </c>
       <c r="B37" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="C37" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="D37" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="E37" t="s">
         <v>35</v>
       </c>
-      <c r="F37" t="s">
-        <v>168</v>
+      <c r="F37" s="4" t="s">
+        <v>164</v>
       </c>
       <c r="G37">
         <v>80</v>
       </c>
       <c r="H37" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.3">
+        <v>129</v>
+      </c>
+      <c r="J37" s="5" t="s">
+        <v>192</v>
+      </c>
+      <c r="K37" s="5"/>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="B38" t="s">
+        <v>165</v>
+      </c>
+      <c r="C38" t="s">
+        <v>166</v>
+      </c>
+      <c r="D38" t="s">
+        <v>167</v>
+      </c>
+      <c r="E38" t="s">
+        <v>168</v>
+      </c>
+      <c r="F38" s="4" t="s">
         <v>169</v>
-      </c>
-      <c r="C38" t="s">
-        <v>170</v>
-      </c>
-      <c r="D38" t="s">
-        <v>171</v>
-      </c>
-      <c r="E38" t="s">
-        <v>172</v>
-      </c>
-      <c r="F38" t="s">
-        <v>173</v>
       </c>
       <c r="G38">
         <v>77</v>
       </c>
       <c r="H38" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.3">
+        <v>73</v>
+      </c>
+      <c r="J38" s="5" t="s">
+        <v>192</v>
+      </c>
+      <c r="K38" s="5"/>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>13</v>
       </c>
       <c r="B39" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="C39" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="D39" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="E39" t="s">
         <v>35</v>
       </c>
-      <c r="F39" t="s">
-        <v>177</v>
+      <c r="F39" s="4" t="s">
+        <v>173</v>
       </c>
       <c r="G39">
         <v>70</v>
       </c>
       <c r="H39" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.3">
+        <v>129</v>
+      </c>
+      <c r="J39" s="5" t="s">
+        <v>192</v>
+      </c>
+      <c r="K39" s="5"/>
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>8</v>
       </c>
       <c r="D40" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="E40" t="s">
         <v>35</v>
       </c>
-      <c r="F40" t="s">
-        <v>179</v>
+      <c r="F40" s="4" t="s">
+        <v>175</v>
       </c>
       <c r="G40">
         <v>70</v>
@@ -2440,25 +2623,29 @@
       <c r="H40" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="J40" s="5" t="s">
+        <v>192</v>
+      </c>
+      <c r="K40" s="5"/>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>13</v>
       </c>
       <c r="B41" t="s">
+        <v>176</v>
+      </c>
+      <c r="C41" t="s">
+        <v>177</v>
+      </c>
+      <c r="D41" t="s">
+        <v>178</v>
+      </c>
+      <c r="E41" t="s">
+        <v>179</v>
+      </c>
+      <c r="F41" s="4" t="s">
         <v>180</v>
-      </c>
-      <c r="C41" t="s">
-        <v>181</v>
-      </c>
-      <c r="D41" t="s">
-        <v>182</v>
-      </c>
-      <c r="E41" t="s">
-        <v>183</v>
-      </c>
-      <c r="F41" t="s">
-        <v>184</v>
       </c>
       <c r="G41">
         <v>65</v>
@@ -2466,80 +2653,131 @@
       <c r="H41" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="J41" s="5" t="s">
+        <v>192</v>
+      </c>
+      <c r="K41" s="5"/>
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>8</v>
       </c>
       <c r="D42" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="E42" t="s">
         <v>35</v>
       </c>
-      <c r="F42" t="s">
-        <v>186</v>
+      <c r="F42" s="4" t="s">
+        <v>182</v>
       </c>
       <c r="G42">
         <v>50</v>
       </c>
       <c r="H42" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.3">
+        <v>107</v>
+      </c>
+      <c r="J42" s="5" t="s">
+        <v>192</v>
+      </c>
+      <c r="K42" s="5"/>
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>13</v>
       </c>
       <c r="B43" t="s">
+        <v>183</v>
+      </c>
+      <c r="C43" t="s">
+        <v>184</v>
+      </c>
+      <c r="D43" t="s">
+        <v>185</v>
+      </c>
+      <c r="E43" t="s">
+        <v>186</v>
+      </c>
+      <c r="F43" s="4" t="s">
         <v>187</v>
-      </c>
-      <c r="C43" t="s">
-        <v>188</v>
-      </c>
-      <c r="D43" t="s">
-        <v>189</v>
-      </c>
-      <c r="E43" t="s">
-        <v>190</v>
-      </c>
-      <c r="F43" t="s">
-        <v>191</v>
       </c>
       <c r="G43">
         <v>55</v>
       </c>
       <c r="H43" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A44" t="s">
-        <v>13</v>
-      </c>
-      <c r="B44" t="s">
-        <v>152</v>
-      </c>
-      <c r="C44" t="s">
-        <v>153</v>
-      </c>
-      <c r="D44" t="s">
+        <v>100</v>
+      </c>
+      <c r="J43" s="5" t="s">
         <v>192</v>
       </c>
-      <c r="E44" t="s">
-        <v>35</v>
-      </c>
-      <c r="F44" t="s">
-        <v>155</v>
-      </c>
-      <c r="G44">
-        <v>50</v>
-      </c>
-      <c r="H44" t="s">
-        <v>133</v>
-      </c>
+      <c r="K43" s="5"/>
+    </row>
+    <row r="44" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="J44" s="2"/>
+      <c r="K44" s="2"/>
     </row>
   </sheetData>
+  <mergeCells count="43">
+    <mergeCell ref="J42:K42"/>
+    <mergeCell ref="J43:K43"/>
+    <mergeCell ref="J44:K44"/>
+    <mergeCell ref="J36:K36"/>
+    <mergeCell ref="J37:K37"/>
+    <mergeCell ref="J38:K38"/>
+    <mergeCell ref="J39:K39"/>
+    <mergeCell ref="J40:K40"/>
+    <mergeCell ref="J41:K41"/>
+    <mergeCell ref="J30:K30"/>
+    <mergeCell ref="J31:K31"/>
+    <mergeCell ref="J32:K32"/>
+    <mergeCell ref="J33:K33"/>
+    <mergeCell ref="J34:K34"/>
+    <mergeCell ref="J35:K35"/>
+    <mergeCell ref="J24:K24"/>
+    <mergeCell ref="J25:K25"/>
+    <mergeCell ref="J26:K26"/>
+    <mergeCell ref="J27:K27"/>
+    <mergeCell ref="J28:K28"/>
+    <mergeCell ref="J29:K29"/>
+    <mergeCell ref="J18:K18"/>
+    <mergeCell ref="J19:K19"/>
+    <mergeCell ref="J20:K20"/>
+    <mergeCell ref="J21:K21"/>
+    <mergeCell ref="J22:K22"/>
+    <mergeCell ref="J23:K23"/>
+    <mergeCell ref="J11:K11"/>
+    <mergeCell ref="J12:K12"/>
+    <mergeCell ref="J13:K13"/>
+    <mergeCell ref="J14:K14"/>
+    <mergeCell ref="J15:K15"/>
+    <mergeCell ref="J16:K16"/>
+    <mergeCell ref="J17:K17"/>
+    <mergeCell ref="J2:K2"/>
+    <mergeCell ref="J3:K3"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="J5:K5"/>
+    <mergeCell ref="J6:K6"/>
+    <mergeCell ref="J7:K7"/>
+    <mergeCell ref="J8:K8"/>
+    <mergeCell ref="J9:K9"/>
+    <mergeCell ref="J10:K10"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="F29" r:id="rId1" xr:uid="{DA7C93E0-2D0C-4A78-A77E-14EF088C67FC}"/>
+    <hyperlink ref="F31" r:id="rId2" xr:uid="{E42EB64A-A1D3-43C7-8C45-364AD6FA1164}"/>
+    <hyperlink ref="F32" r:id="rId3" xr:uid="{55DE9061-98A5-4885-82F0-34FE7D46C6E2}"/>
+    <hyperlink ref="F33" r:id="rId4" xr:uid="{EFA87293-CB01-494C-A6C5-67B68341DB09}"/>
+    <hyperlink ref="F34" r:id="rId5" xr:uid="{F917D0C1-CDD7-4390-9A4B-19D4EAACAF9D}"/>
+    <hyperlink ref="F35" r:id="rId6" xr:uid="{B6D5B62C-A0B8-41E4-9E58-08638EAD2223}"/>
+    <hyperlink ref="F36" r:id="rId7" xr:uid="{CFB3B093-0E30-4951-9C14-D39C51A6A19F}"/>
+    <hyperlink ref="F37" r:id="rId8" xr:uid="{2760417F-31A6-4864-BB4D-8D3DE0EF8C3E}"/>
+    <hyperlink ref="F38" r:id="rId9" xr:uid="{5AE7234D-793E-4B30-B945-C8C3DBA4DDB7}"/>
+    <hyperlink ref="F39" r:id="rId10" xr:uid="{EB58E0C0-E15E-4617-9653-FB6D9B7A7474}"/>
+    <hyperlink ref="F40" r:id="rId11" xr:uid="{42B0DDAC-AAB8-4CF0-BD1B-412401076687}"/>
+    <hyperlink ref="F41" r:id="rId12" xr:uid="{3D1ABECC-F906-47A9-8133-56747DF436BE}"/>
+    <hyperlink ref="F42" r:id="rId13" xr:uid="{D24AAD2A-6C2F-4F5A-987C-C79071F87E57}"/>
+    <hyperlink ref="F43" r:id="rId14" xr:uid="{24575D79-FC4F-40AD-B2AB-B512D9F9BD22}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>